<commit_message>
Atualizacao de agendamento de modulos
</commit_message>
<xml_diff>
--- a/DOCS/Agendamento de modulos.xlsx
+++ b/DOCS/Agendamento de modulos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://radcom365-my.sharepoint.com/personal/rodrigoc_radcom_com/Documents/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodri\iCloudDrive\Development\whatsapp-bot_API\whatsapp-bot_API\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{9F10DE79-4E99-4FA9-9320-9D6E5439E2C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{702AEBA9-DF59-4F77-A144-ED69724B1D7C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA66B12-102F-4176-9FD9-699343D08E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DC3BD5B6-0F0A-48B4-91C2-DE5C5F991C00}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{DC3BD5B6-0F0A-48B4-91C2-DE5C5F991C00}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -80,9 +78,6 @@
     <t>DISPAROS</t>
   </si>
   <si>
-    <t>Clientes com 1 unico pedido entre 7 e 127 dias atras, sem o uso de cupom. (mesmo dis meses anteriores)</t>
-  </si>
-  <si>
     <t>promo_48</t>
   </si>
   <si>
@@ -104,9 +99,6 @@
     <t>recupera_clientes</t>
   </si>
   <si>
-    <t>Clientes que fizeram mais de 2 pedidos e não pedem a 40 dias (mesmo dia meses anteriores)</t>
-  </si>
-  <si>
     <t>satisfação</t>
   </si>
   <si>
@@ -120,6 +112,12 @@
   </si>
   <si>
     <t>~40</t>
+  </si>
+  <si>
+    <t>Clientes com 1 unico pedido há mais de 20 dias atras. (mesmo dis meses anteriores)</t>
+  </si>
+  <si>
+    <t>Clientes que fizeram 2 ou mais pedidos e não pedem a 40 dias (mesmo dia meses anteriores)</t>
   </si>
 </sst>
 </file>
@@ -164,7 +162,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,6 +177,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -211,7 +215,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -232,10 +236,21 @@
     <xf numFmtId="20" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutro" xfId="1" builtinId="28"/>
@@ -572,16 +587,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3951836B-6B1B-4997-B34F-60A14BC00B68}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.88671875" customWidth="1"/>
-    <col min="2" max="2" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="8" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="86.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="86.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -610,10 +625,10 @@
         <v>13</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -627,9 +642,9 @@
       <c r="I2" s="4"/>
       <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -641,9 +656,9 @@
       <c r="I3" s="4"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="7">
@@ -658,10 +673,10 @@
         <v>20</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -675,13 +690,13 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
@@ -695,13 +710,13 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
@@ -728,42 +743,42 @@
         <v>21</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="8" t="s">
+      <c r="J8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="2" t="s">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="5">
@@ -787,43 +802,43 @@
       <c r="I9" s="6">
         <v>24</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="13">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="C10" s="13">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="D10" s="13">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="E10" s="13">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="F10" s="13">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="G10" s="13">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="H10" s="13">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="I10" s="14"/>
+      <c r="J10" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="5">
-        <v>0.43194444444444446</v>
-      </c>
-      <c r="C10" s="5">
-        <v>0.43194444444444446</v>
-      </c>
-      <c r="D10" s="5">
-        <v>0.43194444444444446</v>
-      </c>
-      <c r="E10" s="5">
-        <v>0.43194444444444446</v>
-      </c>
-      <c r="F10" s="5">
-        <v>0.43194444444444446</v>
-      </c>
-      <c r="G10" s="5">
-        <v>0.43194444444444446</v>
-      </c>
-      <c r="H10" s="5">
-        <v>0.43194444444444446</v>
-      </c>
-      <c r="I10" s="4"/>
-      <c r="J10" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -835,8 +850,8 @@
       <c r="I11" s="4"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="G13" s="9"/>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G13" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>